<commit_message>
feat: projectile과 paritcleComponent 삭제 흐름 수정
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/PetActiveSkillData.xlsx
+++ b/JsonConverter/ExcelFiles/PetActiveSkillData.xlsx
@@ -164,7 +164,7 @@
     <t>Fire</t>
   </si>
   <si>
-    <t>FramePawn/ActiveEffect</t>
+    <t>FramePawn_ActiveEffect</t>
   </si>
   <si>
     <t>pet_skill_water_001</t>
@@ -179,7 +179,7 @@
     <t>Cold</t>
   </si>
   <si>
-    <t>WaterPawn/ActiveEffect</t>
+    <t>WaterPawn_ActiveEffect</t>
   </si>
   <si>
     <t>pet_skill_earth_001</t>
@@ -197,7 +197,7 @@
     <t>Physical</t>
   </si>
   <si>
-    <t>EarthPawn/ActiveEffect</t>
+    <t>EarthPawn_ActiveEffect</t>
   </si>
   <si>
     <t>pet_skill_air_001</t>
@@ -209,7 +209,7 @@
     <t>관통하지 않는 빠른 바람 투사체를 발사해 단일 적에게 물리 피해를 줍니다. 기본 공격 자체는 상태이상을 부여하지 않습니다.</t>
   </si>
   <si>
-    <t>WindPawn/ActiveEffect</t>
+    <t>WindPawn_ActiveEffect</t>
   </si>
   <si>
     <t>pet_skill_taunt</t>
@@ -332,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -367,10 +367,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="0"/>
@@ -940,7 +943,7 @@
       <c r="L6" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="M6" s="11" t="s">
+      <c r="M6" s="13" t="s">
         <v>59</v>
       </c>
       <c r="N6" s="8" t="s">
@@ -1042,7 +1045,7 @@
       <c r="L8" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="M8" s="11" t="s">
+      <c r="M8" s="13" t="s">
         <v>70</v>
       </c>
       <c r="N8" s="8"/>
@@ -1094,7 +1097,7 @@
       <c r="N9" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="O9" s="11" t="s">
+      <c r="O9" s="13" t="s">
         <v>78</v>
       </c>
       <c r="P9" s="8"/>
@@ -5706,25 +5709,25 @@
       <c r="T218" s="12"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
-      <c r="A219" s="13"/>
-      <c r="B219" s="13"/>
-      <c r="C219" s="13"/>
-      <c r="D219" s="14"/>
-      <c r="E219" s="13"/>
-      <c r="F219" s="13"/>
-      <c r="G219" s="14"/>
-      <c r="H219" s="13"/>
-      <c r="I219" s="13"/>
-      <c r="J219" s="13"/>
-      <c r="K219" s="15"/>
-      <c r="L219" s="13"/>
-      <c r="M219" s="13"/>
-      <c r="N219" s="13"/>
-      <c r="O219" s="13"/>
-      <c r="P219" s="13"/>
-      <c r="Q219" s="13"/>
-      <c r="R219" s="14"/>
-      <c r="S219" s="14"/>
+      <c r="A219" s="14"/>
+      <c r="B219" s="14"/>
+      <c r="C219" s="14"/>
+      <c r="D219" s="15"/>
+      <c r="E219" s="14"/>
+      <c r="F219" s="14"/>
+      <c r="G219" s="15"/>
+      <c r="H219" s="14"/>
+      <c r="I219" s="14"/>
+      <c r="J219" s="14"/>
+      <c r="K219" s="16"/>
+      <c r="L219" s="14"/>
+      <c r="M219" s="14"/>
+      <c r="N219" s="14"/>
+      <c r="O219" s="14"/>
+      <c r="P219" s="14"/>
+      <c r="Q219" s="14"/>
+      <c r="R219" s="15"/>
+      <c r="S219" s="15"/>
       <c r="T219" s="12"/>
     </row>
     <row r="220" ht="15.75" customHeight="1">

</xml_diff>